<commit_message>
Correct preferential-origin conclusion and add JSD field check
Verified against Regulation (EU) 2025/1909: India is graduated out of
GSP section S-13 (chapters 68-70, glass) from 1 Jan 2026 to 31 Dec 2028.
HS 7019 90 00 falls in S-13, so the REX statement on the invoice cannot
be used and preference code 100 (erga omnes) is correct - this reverses
the earlier note that told the user to claim GSP.

Also:
- New "Kontrola JSD" sheet checking the declaration screen field by
  field; country of origin CN is wrong and must be IN
- Anti-dumping note sharpened: 2020/492 and 2020/776 target TARIC line
  7019 90 00 80 for CN/EG origin; line 85 with IN origin is outside it
- Box 31 description does not match the invoice wording, proposed text

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YQQ8xTARGbCQADaJcoDAot
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_2JCP_CZ26012407.xlsx
+++ b/output/HS_Code_Summary_2JCP_CZ26012407.xlsx
@@ -10,6 +10,7 @@
     <sheet name="HS Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Položky faktury" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Poznámky a kontroly" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Kontrola JSD" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -52,7 +53,7 @@
       <color rgb="001F3864"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -71,12 +72,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFE699"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -106,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -147,6 +153,15 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -512,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -616,305 +631,329 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Indie (IN)</t>
+          <t>INDIE (IN) – POZOR: nikoli CN! Faktura: „Country of origin of goods: India“, REX prohlášení zní na „INDIA“, nakládka Chennai.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Země určení:</t>
+          <t>Zbožový kód:</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Česká republika (CZ)</t>
+          <t>7019 90 00, TARIC 7019 90 00 85 (ostatní) – dle faktury a B/L; kód preference 100 (erga omnes), viz preferenční blok níže</t>
         </is>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Incoterm:</t>
+          <t>Země určení:</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>EXW Chennai (Indie) – dle faktury „Terms of Delivery: EXW“, místo nakládky Chennai</t>
+          <t>Česká republika (CZ)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Měna:</t>
+          <t>Incoterm:</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>DKK (dánská koruna) – přepočet na CZK celním kurzem platným pro měsíc podání JSD</t>
+          <t>EXW Chennai (Indie) – dle faktury „Terms of Delivery: EXW“, místo nakládky Chennai</t>
         </is>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>Měna:</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>DKK (dánská koruna) – přepočet na CZK celním kurzem platným pro měsíc podání JSD</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>Očekávaný příchod:</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>ECU WORLDWIDE (CZ) s.r.o., Hrušov – cca 20. 9. 2026, dle e-mailu bude SCP</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="34" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Odesílatel</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>HS kód</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Popis zboží (dle faktury)</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Popis zboží (CZ)</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>Země původu</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>Množství (ks)</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>Čistá hmotnost (kg)</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>Hrubá hmotnost (kg)</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>Hodnota zboží (DKK)</t>
         </is>
       </c>
-      <c r="J15" s="4" t="inlineStr">
+      <c r="J16" s="4" t="inlineStr">
         <is>
           <t>Balné (DKK)</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr">
+      <c r="K16" s="4" t="inlineStr">
         <is>
           <t>Celní hodnota – základ (DKK)</t>
         </is>
       </c>
-      <c r="L15" s="4" t="inlineStr">
+      <c r="L16" s="4" t="inlineStr">
         <is>
           <t>Poznámka</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="90" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
+    <row r="17" ht="90" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>EagleBurgmann KE Private Limited, Chennai, Indie</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>70199000</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>Non Metalic Expansion Joint (Fabric Expansion Joint, Bolster Type 66, Steel Foil HF, Wiremesh 16/16, KE Pulse Breaker A, KE1400 HT, Joining Kit)</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>Nekovové kompenzátory ze skleněných vláken – tkaninové kompenzátory, izolační vložky (bolstery), ocelové fólie, drátěné síťoviny, tlumič pulzací, spojovací sady</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="F16" s="6" t="n">
+      <c r="F17" s="6" t="n">
         <v>35</v>
       </c>
-      <c r="G16" s="7" t="n">
+      <c r="G17" s="7" t="n">
         <v>1180</v>
       </c>
-      <c r="H16" s="7" t="n">
+      <c r="H17" s="7" t="n">
         <v>1420</v>
       </c>
-      <c r="I16" s="8" t="n">
+      <c r="I17" s="8" t="n">
         <v>207779.39</v>
       </c>
-      <c r="J16" s="8" t="n">
+      <c r="J17" s="8" t="n">
         <v>5450</v>
       </c>
-      <c r="K16" s="8" t="n">
+      <c r="K17" s="8" t="n">
         <v>213229.39</v>
       </c>
-      <c r="L16" s="5" t="inlineStr">
+      <c r="L17" s="5" t="inlineStr">
         <is>
           <t>Jediný HS kód dle faktury a B/L (HS Tariff 70 19 90 00). Balné 5 450 DKK je součástí celní hodnoty (čl. 71 UCC). K celní hodnotě nutno přičíst dopravné do místa vstupu do EU – EXW + freight collect (viz list „Poznámky a kontroly“).</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>CELKEM</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr"/>
-      <c r="C17" s="9" t="inlineStr"/>
-      <c r="D17" s="9" t="inlineStr"/>
-      <c r="E17" s="9" t="inlineStr"/>
-      <c r="F17" s="10" t="n">
+      <c r="B18" s="9" t="inlineStr"/>
+      <c r="C18" s="9" t="inlineStr"/>
+      <c r="D18" s="9" t="inlineStr"/>
+      <c r="E18" s="9" t="inlineStr"/>
+      <c r="F18" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="G17" s="11" t="n">
+      <c r="G18" s="11" t="n">
         <v>1180</v>
       </c>
-      <c r="H17" s="11" t="n">
+      <c r="H18" s="11" t="n">
         <v>1420</v>
       </c>
-      <c r="I17" s="12" t="n">
+      <c r="I18" s="12" t="n">
         <v>207779.39</v>
       </c>
-      <c r="J17" s="12" t="n">
+      <c r="J18" s="12" t="n">
         <v>5450</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="K18" s="12" t="n">
         <v>213229.39</v>
       </c>
-      <c r="L17" s="9" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+      <c r="L18" s="9" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
         <is>
           <t>PŘÍZNAKY A KONTROLY</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="62" customHeight="1">
-      <c r="A20" s="13" t="inlineStr">
-        <is>
-          <t>🟢 PREFERENČNÍ VĚTA – ANO</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Na faktuře je uvedeno preferenční prohlášení (REX): „The exporter Ms. EagleBurgmann KE Pvt. Ltd., REX Registration No.: INREX0500068909EC013 of the products covered by this document declares that, except where otherwise clearly indicated, these products are of "INDIA" preferential origin according to rules of origin of the Generalized System of Preferences of the European Union and that the origin criterion met is "W" [Heading of HS System: 7019].“ → Uplatnit preferenční celní sazbu GSP pro Indii místo standardní sazby erga omnes. KRITICKÉ pro správné vyclení – ověřit platnost REX čísla v databázi REX a sazbu v TARIC ke dni přijetí JSD.</t>
-        </is>
-      </c>
-    </row>
     <row r="21" ht="62" customHeight="1">
-      <c r="A21" s="14" t="inlineStr">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>🔴 PREFERENČNÍ VĚTA JE, ALE PREFERENCI NELZE UPLATNIT</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Na faktuře JE preferenční prohlášení (REX): „The exporter Ms. EagleBurgmann KE Pvt. Ltd., REX Registration No.: INREX0500068909EC013 … these products are of "INDIA" preferential origin according to rules of origin of the Generalized System of Preferences of the European Union … origin criterion "W" [Heading of HS System: 7019].“ ALE: Indie je od 1. 1. 2026 do 31. 12. 2028 vyřazena (graduace) ze sekce GSP S-13 „Výrobky z kamene, sádry, cementu, azbestu, slídy; keramické výrobky; SKLO“ (kap. 68–70) dle nařízení (EU) 2025/1909. Kód 7019 90 00 spadá do S-13 → pro původ IN NENÍ v roce 2026 dostupná preference GSP. → Uplatní se standardní sazba třetích zemí, kód preference 100. Prohlášení REX ponechat ve spisu, ale preferenci NENÁROKOVAT. Ověřit v TARIC ke dni přijetí JSD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="62" customHeight="1">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>🔴 JSD – ZEMĚ PŮVODU</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>V celním prohlášení musí být země původu IN (Indie), NIKOLI CN (Čína). Původ CN by byl nesprávnou deklarací a navíc by u kap. 7019 mohl aktivovat antidumpingová/vyrovnávací opatření na skleněná vlákna z ČLR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="62" customHeight="1">
+      <c r="A23" s="14" t="inlineStr">
         <is>
           <t>⚪ CBAM – netýká se</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>HS 7019 90 00 (výrobky ze skleněných vláken) není zbožím podle přílohy I nařízení CBAM (cement, železo a ocel, hliník, hnojiva, elektřina, vodík). CBAM kód se v této zásilce neuvádí. Pozn.: příjemce 2JCP a.s. ani EagleBurgmann KE A/S NEJSOU v registru reference/CBAM_receivers_CZ.xlsx – pokud by v budoucí zásilce bylo CBAM zboží, je nutné firmu prověřit a do registru doplnit.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="62" customHeight="1">
-      <c r="A22" s="14" t="inlineStr">
+    <row r="24" ht="62" customHeight="1">
+      <c r="A24" s="14" t="inlineStr">
         <is>
           <t>⚪ Antidumping – dle původu se nepředpokládá</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Antidumpingová/vyrovnávací opatření EU na výrobky ze skleněných vláken (kap. 7019) se vztahují na původ ČLR a Egypt. Původ tohoto zboží je INDIE, opatření by se tedy uplatnit neměla. Přesto ověřit v TARIC pro kód 7019 90 00 / původ IN ke dni podání JSD.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="62" customHeight="1">
-      <c r="A23" s="15" t="inlineStr">
-        <is>
-          <t>🟡 Celní hodnota – dopravné</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Dodací podmínka EXW Chennai, přeprava „freight collect“, všechny náklady v destinaci hrazeny při dodání. Do celní hodnoty je nutno připočíst náklady dopravy a pojištění až na místo vstupu do EU (Hamburk). Vyžádat si od ECU Worldwide / Maurice Ward rozpis přepravného.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="62" customHeight="1">
-      <c r="A24" s="15" t="inlineStr">
-        <is>
-          <t>🟡 Clení v dánském EORI</t>
-        </is>
-      </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Dle pokynu zákazníka má být zásilka vyclena na dánské EORI EagleBurgmann (EagleBurgmann KE A/S, Dánsko) jako obvykle, ačkoli zboží fyzicky míří k 2JCP a.s. v ČR. Ověřit platnou plnou moc (nepřímé zastoupení) a DPH režim dovozu v ČR pro subjekt neusazený v ČR.</t>
+          <t>Antidumpingová a vyrovnávací opatření EU na tkaniny ze skleněných vláken (nař. (EU) 2020/492 a 2020/776) se týkají původu ČLR a Egypt a v rámci 7019 90 00 míří na TARIC linku …80. Zde je původ INDIE a použita TARIC linka …85 (ostatní) → opatření se neuplatní. Ověřit v TARIC pro 7019 90 00 85 / původ IN ke dni podání JSD.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="62" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>🟡 Rozpor v adrese příjemce</t>
+          <t>🟡 Celní hodnota – dopravné</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Faktura/packing list uvádí 2JCP, Průmyslová 162, 674 01 Třebíč; HBL uvádí 2JCP, Račice 126, 411 08 Štětí. Před podáním JSD potvrdit správnou adresu (a EORI) příjemce.</t>
+          <t>Dodací podmínka EXW Chennai, přeprava „freight collect“, všechny náklady v destinaci hrazeny při dodání. Do celní hodnoty je nutno připočíst náklady dopravy a pojištění až na místo vstupu do EU (Hamburk). Vyžádat si od ECU Worldwide / Maurice Ward rozpis přepravného.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="62" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
+          <t>🟡 Clení v dánském EORI</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Dle pokynu zákazníka má být zásilka vyclena na dánské EORI EagleBurgmann (EagleBurgmann KE A/S, Dánsko) jako obvykle, ačkoli zboží fyzicky míří k 2JCP a.s. v ČR. Ověřit platnou plnou moc (nepřímé zastoupení) a DPH režim dovozu v ČR pro subjekt neusazený v ČR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="62" customHeight="1">
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t>🟡 Rozpor v adrese příjemce</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Faktura/packing list uvádí 2JCP, Průmyslová 162, 674 01 Třebíč; HBL uvádí 2JCP, Račice 126, 411 08 Štětí. Před podáním JSD potvrdit správnou adresu (a EORI) příjemce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="62" customHeight="1">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
           <t>🟡 Rozpor v packing listu</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>Rozpis balení na packing listu uvádí „Pulse Breaker – 5 PC“, zatímco Annexure-I obsahuje 1 ks KE Pulse Breaker A. Součet položek Annexure-I = 35 ks a odpovídá deklarovanému celkovému množství 35 ks; rozpis v packing listu (39 ks) je zjevně chybný. Pro JSD použito množství dle Annexure-I.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="62" customHeight="1">
-      <c r="A27" s="14" t="inlineStr">
+    <row r="29" ht="62" customHeight="1">
+      <c r="A29" s="14" t="inlineStr">
         <is>
           <t>⚪ Sleva</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>Na faktuře není uvedena žádná obchodní sleva – proporcionální rozpouštění slevy se neuplatní.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="22">
     <mergeCell ref="B4:L4"/>
     <mergeCell ref="B26:L26"/>
     <mergeCell ref="B7:L7"/>
@@ -925,16 +964,18 @@
     <mergeCell ref="B12:L12"/>
     <mergeCell ref="B21:L21"/>
     <mergeCell ref="B11:L11"/>
+    <mergeCell ref="B14:L14"/>
     <mergeCell ref="B23:L23"/>
     <mergeCell ref="B8:L8"/>
     <mergeCell ref="B13:L13"/>
+    <mergeCell ref="B29:L29"/>
     <mergeCell ref="B10:L10"/>
+    <mergeCell ref="B28:L28"/>
     <mergeCell ref="B9:L9"/>
     <mergeCell ref="B6:L6"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="B24:L24"/>
     <mergeCell ref="B5:L5"/>
-    <mergeCell ref="B20:L20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1958,7 +1999,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A56"/>
+  <dimension ref="A1:A62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -1973,14 +2014,14 @@
     <row r="2">
       <c r="A2" s="21" t="inlineStr">
         <is>
-          <t>NA FAKTUŘE JE PREFERENČNÍ VĚTA (prohlášení o původu REX) – uplatnit preferenci!</t>
+          <t>PREFERENČNÍ VĚTA NA FAKTUŘE JE – ale preferenci pro rok 2026 NELZE uplatnit. Uplatní se kód preference 100.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Znění: „REX Declaration: The exporter Ms. EagleBurgmann KE Pvt. Ltd., REX Registration No.: INREX0500068909EC013 of the</t>
+          <t>Znění na faktuře: „REX Declaration: The exporter Ms. EagleBurgmann KE Pvt. Ltd., REX Registration No.: INREX0500068909EC013 of the</t>
         </is>
       </c>
     </row>
@@ -2006,315 +2047,357 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>→ Dopad: bez tohoto prohlášení by se uplatnila standardní sazba třetích zemí. S platným prohlášením lze uplatnit</t>
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>DŮVOD, PROČ PREFERENCE NEPLATÍ:</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">   preferenční sazbu GSP pro Indii (snížené / nulové clo).</t>
+          <t>Indie byla nařízením (EU) 2025/1909 vyřazena (graduace) ze sekce GSP S-13 = „Výrobky z kamene, sádry, cementu, azbestu,</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>→ Před podáním JSD ověřit: platnost REX čísla INREX0500068909EC013 v databázi REX EU a preferenční sazbu</t>
+          <t>slídy nebo podobných materiálů; keramické výrobky; SKLO A SKLENĚNÉ VÝROBKY“ (kapitoly 68–70), a to na období</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">   pro 7019 90 00 / původ IN v TARIC ke dni přijetí celního prohlášení.</t>
+          <t>od 1. 1. 2026 do 31. 12. 2028. Zbožový kód 7019 90 00 je kapitola 70 → spadá do S-13 → GSP preference pro původ IN</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>→ Pozn.: vývozce je registrovaný vývozce (REX), hodnota zásilky přesahuje 6 000 EUR – prohlášení je proto formálně v pořádku.</t>
+          <t>v tomto období NENÍ dostupná. Prohlášení REX je tedy formálně platné, ale bez celního dopadu.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>→ V JSD uvést kód preference 100 (erga omnes / standardní sazba třetích zemí), NIKOLI 200 (GSP).</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="21">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>→ Prohlášení REX přesto založit do spisu k zásilce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>→ Sazbu erga omnes pro 7019 90 00 85 ověřit v TARIC / e-Dovoz ke dni přijetí celního prohlášení.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>→ Pozn.: u dřívějších zásilek EagleBurgmann Indie (do 31. 12. 2025) preference GSP dostupná byla – od 1. 1. 2026 už ne.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="21">
         <f>== CBAM ===</f>
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>HS 7019 90 00 = výrobky ze skleněných vláken → NENÍ zboží podle přílohy I nařízení CBAM. CBAM se na tuto zásilku nevztahuje.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Kontrola registru reference/CBAM_receivers_CZ.xlsx (list List1): ani „2JCP a.s.“, ani „EagleBurgmann KE A/S“ v registru NEJSOU.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>→ Pro tuto zásilku to nevadí (CBAM zboží zde není). Pokud však u některé příští zásilky bude CBAM zboží,</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t xml:space="preserve">   je nutné firmu prověřit a doplnit do registru včetně Y kódu (Y128 / Y238 / Y137).</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="21">
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="21">
         <f>== ANTIDUMPING ===</f>
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Antidumpingová a vyrovnávací opatření EU u kapitoly 7019 (skleněná vlákna, rovingy, tkaniny) míří na původ ČLR a Egypt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Původ zboží v této zásilce je INDIE → opatření by se uplatnit neměla. Ověřit v TARIC (kód 7019 90 00, původ IN) při podání JSD.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="21">
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Antidumpingová a vyrovnávací opatření EU na tkaniny ze skleněných vláken (nař. (EU) 2020/492, 2020/776) se týkají původu ČLR a Egypt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>V rámci 7019 90 00 míří tato opatření na TARIC linku 7019 90 00 80. Zde je použita linka 7019 90 00 85 (ostatní) a původ INDIE →</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>opatření se neuplatní. Právě proto je volba TARIC linky 85 (ne 80) podstatná. Ověřit v TARIC při podání JSD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>POZOR: kdyby v JSD zůstal původ CN, TARIC by u kap. 7019 mohl vyžadovat antidumpingový přídavný kód – další důvod původ opravit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="21">
         <f>== INCOTERM ===</f>
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t>EXW Chennai (Indie) – dle faktury „Terms of Delivery &amp; Payment: EXW“, místo převzetí / přístav nakládky Chennai.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
+    <row r="31">
+      <c r="A31" t="inlineStr">
         <is>
           <t>Přeprava LCL/LCL, „FREIGHT COLLECT“, všechny náklady v destinaci hrazeny při dodání (MBL i HBL).</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
+    <row r="32">
+      <c r="A32" t="inlineStr">
         <is>
           <t>→ Do celní hodnoty připočíst dopravné + pojištění až do místa vstupu do EU (přístav vykládky Hamburk).</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>→ Vyžádat rozpis přepravních nákladů od ECU Worldwide (CZ) / Maurice Ward.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="21">
+    <row r="34">
+      <c r="A34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="21">
         <f>== HODNOTY A HMOTNOSTI ===</f>
         <v/>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Hodnota zboží dle faktury č. 266: 207 779,39 DKK (35 ks, součet Annexure-I ověřen).</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Balné (Packing Charges): 5 450,00 DKK – dle čl. 71 UCC součást celní hodnoty.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Fakturovaná částka celkem: 213 229,39 DKK.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Obchodní sleva: žádná (na faktuře neuvedena) → proporcionální rozpuštění slevy se neuplatňuje.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Čistá hmotnost: 1 180,00 kg; hrubá hmotnost: 1 420,00 kg (shodně faktura/packing list, MBL i HBL). Objem 10,098 m³.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Vše pod jedním HS kódem → rozpouštění hmotností a hodnot mezi kódy není potřeba.</t>
-        </is>
-      </c>
-    </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>Hodnota zboží dle faktury č. 266: 207 779,39 DKK (35 ks, součet Annexure-I ověřen).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Balné (Packing Charges): 5 450,00 DKK – dle čl. 71 UCC součást celní hodnoty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Fakturovaná částka celkem: 213 229,39 DKK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Obchodní sleva: žádná (na faktuře neuvedena) → proporcionální rozpuštění slevy se neuplatňuje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Čistá hmotnost: 1 180,00 kg; hrubá hmotnost: 1 420,00 kg (shodně faktura/packing list, MBL i HBL). Objem 10,098 m³.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Vše pod jedním HS kódem → rozpouštění hmotností a hodnot mezi kódy není potřeba.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>Přepočet DKK → CZK proveďte celním kurzem platným pro měsíc přijetí celního prohlášení.</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="21">
+    <row r="43">
+      <c r="A43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="21">
         <f>== ROZPORY V DOKLADECH – OVĚŘIT ===</f>
         <v/>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
+    <row r="45">
+      <c r="A45" t="inlineStr">
         <is>
           <t>1) Adresa příjemce: faktura + packing list = 2JCP, Průmyslová 162, 674 01 Třebíč; HBL = 2JCP, Račice 126, 411 08 Štětí.</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
+    <row r="46">
+      <c r="A46" t="inlineStr">
         <is>
           <t>2) Packing list uvádí „Pulse Breaker – 5 PC“, ale Annexure-I obsahuje 1 ks. Součet Annexure-I = 35 ks = deklarovaný celkový počet;</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
+    <row r="47">
+      <c r="A47" t="inlineStr">
         <is>
           <t xml:space="preserve">   rozpis v packing listu by dával 39 ks. Pro JSD použito množství dle Annexure-I (35 ks).</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
+    <row r="48">
+      <c r="A48" t="inlineStr">
         <is>
           <t>3) MBL uvádí přístav vykládky Hamburk a místo dodání Praha; HBL uvádí Prague/Prague. Fyzická dodávka dle e-mailu:</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
+    <row r="49">
+      <c r="A49" t="inlineStr">
         <is>
           <t xml:space="preserve">   ECU Worldwide (CZ) s.r.o., Hrušov, cca 20. 9. 2026.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="21">
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="21">
         <f>== CLENÍ / ZASTOUPENÍ ===</f>
         <v/>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
+    <row r="52">
+      <c r="A52" t="inlineStr">
         <is>
           <t>Dle e-mailu Moniky Karlíkové (Maurice Ward): „Clení by mělo být provedeno v dánském čísle EORI EagleBurgmann jako obvykle.“</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
+    <row r="53">
+      <c r="A53" t="inlineStr">
         <is>
           <t>Deklarant/dovozce = EagleBurgmann KE A/S, Odinsvej 1, 6950 Ringkøbing, Dánsko (na faktuře jako „Bill To“).</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
+    <row r="54">
+      <c r="A54" t="inlineStr">
         <is>
           <t>Zboží fyzicky dodáno k 2JCP a.s. v ČR („Ship To“) → řetězový obchod.</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
+    <row r="55">
+      <c r="A55" t="inlineStr">
         <is>
           <t>→ Ověřit platnou plnou moc (nepřímé zastoupení) a režim DPH při dovozu v ČR pro subjekt neusazený v ČR.</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="21">
+    <row r="56">
+      <c r="A56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="21">
         <f>== POUŽITÉ DOKLADY ===</f>
         <v/>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
+    <row r="58">
+      <c r="A58" t="inlineStr">
         <is>
           <t>• Commercial Invoice + Packing List + Annexure-I č. 266 ze dne 9. 7. 2026 (DK26000863_com_inv.pdf)</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
+    <row r="59">
+      <c r="A59" t="inlineStr">
         <is>
           <t>• Master B/L MAA/PRG/01684, Allcargo Global Ltd, vydán 22. 7. 2026 (DK26000863_MBL.pdf)</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
+    <row r="60">
+      <c r="A60" t="inlineStr">
         <is>
           <t>• House B/L (MTD) SEF/MAA/000013/26-27, CCI Worldwide Logistics, Chennai 22. 7. 2026 (DK26000863_HBL.pdf)</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
+    <row r="61">
+      <c r="A61" t="inlineStr">
         <is>
           <t>• E-mail Monika Karlíková, Maurice Ward, věc OR/Import/CZ26012407/2JCP,a.s.</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
+    <row r="62">
+      <c r="A62" t="inlineStr">
         <is>
           <t>• Pokyn ze zadání: „Popis + HS code prosím použít z faktury.“ → použit HS 70 19 90 00 a popisy z faktury.</t>
         </is>
@@ -2323,4 +2406,413 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="78" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Kontrola vyplnění celního prohlášení (list 1 – Běžné údaje) proti dokladům</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Kolonka / pole</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Zadáno v JSD</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Má být</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Stav</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Zdůvodnění / zdroj</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="58" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>34. Země původu (Z.původu)</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="D4" s="22" t="inlineStr">
+        <is>
+          <t>CHYBA</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Faktura, kol. „Country of origin of goods: India“; REX prohlášení zní na „INDIA“; nakládka Chennai, Indie. CN (Čína) je nesprávný původ a u kap. 7019 může navíc aktivovat antidumpingová opatření.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="58" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>36. Kód preference</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="D5" s="23" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Správně. Preferenční věta REX na faktuře sice je, ale Indie je nař. (EU) 2025/1909 od 1. 1. 2026 do 31. 12. 2028 vyřazena ze sekce GSP S-13 (kap. 68–70, sklo). Pro 7019 90 00 tedy preference GSP neplatí → erga omnes, kód 100. Kód 200 (GSP) NEUVÁDĚT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>33. Zbožový kód</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>70199000</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>70199000</t>
+        </is>
+      </c>
+      <c r="D6" s="23" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Odpovídá faktuře („HS Tariff: 70 19 90 00“) i B/L („HS CODE: 70199000“) a pokynu zákazníka použít HS kód z faktury.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="58" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>33. TARIC (DK)</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="D7" s="23" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>7019 90 00 85 = „ostatní“. Linka 7019 90 00 80 je ta, na kterou míří antidumping na tkaniny ze skleněných vláken (ČLR/Egypt) – volba 85 je zde správná.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="58" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>31. Popis zboží</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Termoizolační návleky ze skelného vlákna, kompenzátory, bolstery, ocelové fólie, síťoviny, spojovací sady / 35ks</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Nekovové kompenzátory ze skleněných vláken (tkaninové kompenzátory, izolační vložky – bolstery, ocelové fólie, drátěné síťoviny, tlumič pulzací, spojovací sady), 35 ks, 1 dřevěná bedna, zn. DEN01029/26</t>
+        </is>
+      </c>
+      <c r="D8" s="24" t="inlineStr">
+        <is>
+          <t>UPRAVIT</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Faktura zní „Non Metalic Expansion Joint“ = nekovový kompenzátor. „Termoizolační návleky“ neodpovídá popisu na faktuře – popis by měl odpovídat dokladům a odůvodňovat zařazení. Doplnit značky/počet kusů obalu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="58" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Č.p. (položka)</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D9" s="23" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Jediný HS kód, jediný odesílatel → jedna položka.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="58" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Množství</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>35 ks</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>35 ks</t>
+        </is>
+      </c>
+      <c r="D10" s="23" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Annexure-I: součet 35 ks; faktura i packing list uvádějí celkem 35. (Rozpis v packing listu „Pulse Breaker – 5 PC“ je chybný, dával by 39.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="58" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Kód CH / metoda hodnoty</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>1 – Metoda 1</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>1 – Metoda 1</t>
+        </is>
+      </c>
+      <c r="D11" s="23" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Transakční hodnota – běžný prodej mezi EagleBurgmann Indie a EagleBurgmann KE A/S. OK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="58" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>37. Režim / upřesnění</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>000</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>000 (režim 40 00)</t>
+        </is>
+      </c>
+      <c r="D12" s="24" t="inlineStr">
+        <is>
+          <t>OVĚŘIT</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Volný oběh bez zvláštností je v pořádku. Protože se clí na dánské EORI EagleBurgmann KE A/S (subjekt neusazený v ČR) a zboží zůstává v ČR u 2JCP, ověřit režim DPH a platnou plnou moc k nepřímému zastoupení.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="58" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>38./35. Hmotnosti</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>(není na snímku)</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Čistá 1 180,00 kg / hrubá 1 420,00 kg</t>
+        </is>
+      </c>
+      <c r="D13" s="24" t="inlineStr">
+        <is>
+          <t>DOPLNIT</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Shodně faktura, packing list, MBL i HBL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="58" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>42./45./46. Celní hodnota</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>(není na snímku)</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Zboží 207 779,39 DKK + balné 5 450,00 DKK + dopravné do vstupu do EU</t>
+        </is>
+      </c>
+      <c r="D14" s="24" t="inlineStr">
+        <is>
+          <t>DOPLNIT</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>EXW Chennai + freight collect → dopravné a pojištění do místa vstupu do EU (Hamburk) je nutno k celní hodnotě přičíst. Balné je součástí celní hodnoty (čl. 71 UCC). Přepočet DKK→CZK celním kurzem měsíce přijetí JSD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="58" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>20. Dodací podmínka</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>(není na snímku)</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>EXW Chennai</t>
+        </is>
+      </c>
+      <c r="D15" s="24" t="inlineStr">
+        <is>
+          <t>DOPLNIT</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Faktura: „Terms of Delivery &amp; Payment: EXW“, místo převzetí / přístav nakládky Chennai.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="58" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>8. Příjemce</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>(není na snímku)</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Ověřit adresu 2JCP</t>
+        </is>
+      </c>
+      <c r="D16" s="24" t="inlineStr">
+        <is>
+          <t>OVĚŘIT</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Faktura/packing list: Průmyslová 162, 674 01 Třebíč. HBL: Račice 126, 411 08 Štětí. Před podáním sjednotit.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>